<commit_message>
Second audit pass on Clase 4 (MCO); add el_pct to descriptives; update cronograma
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Cronograma_Analisis_Econometrico_2026.xlsx
+++ b/Cronograma_Analisis_Econometrico_2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ramirodeelejalde/Dropbox/Teaching/Econometria I_MAE/econometria_mae/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{696C346F-0FDA-474A-A158-33C47AAD97B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{999CF562-A876-1F40-AE4D-DDED07E37B6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="440" yWindow="1080" windowWidth="24860" windowHeight="15680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7740" yWindow="1680" windowWidth="24860" windowHeight="15680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cronograma" sheetId="1" r:id="rId1"/>
@@ -124,9 +124,6 @@
     <t xml:space="preserve">Presentación Trabajo Grupal </t>
   </si>
   <si>
-    <t>Trabajo Grupal</t>
-  </si>
-  <si>
     <t>Ayudantía 2: Control 1/ Solución tarea 1</t>
   </si>
   <si>
@@ -167,6 +164,9 @@
   </si>
   <si>
     <t xml:space="preserve">Ayudante 2026: Alexis Silva. Horario por confirmar. </t>
+  </si>
+  <si>
+    <t>Trabajo Grupal/Presentación</t>
   </si>
 </sst>
 </file>
@@ -356,10 +356,6 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="3" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="16" fontId="4" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="4" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
@@ -372,6 +368,10 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="3" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -599,38 +599,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27" t="s">
+      <c r="B1" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="27" t="s">
+      <c r="C1" s="39" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="27" t="s">
+      <c r="D1" s="39" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1"/>
-      <c r="G1" s="27" t="s">
+      <c r="G1" s="39" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="28"/>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
+      <c r="A2" s="40"/>
+      <c r="B2" s="40"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
       <c r="E2" s="2" t="s">
         <v>6</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="28"/>
+      <c r="G2" s="40"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="8">
@@ -682,7 +682,7 @@
       <c r="E5" s="6"/>
       <c r="F5" s="6"/>
       <c r="G5" s="7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -732,7 +732,7 @@
         <v>46268</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E8" s="15"/>
       <c r="F8" s="12"/>
@@ -772,75 +772,75 @@
       <c r="F10" s="10"/>
       <c r="G10" s="25"/>
     </row>
-    <row r="11" spans="1:7" s="37" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="34">
+    <row r="11" spans="1:7" s="35" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="32">
         <v>3</v>
       </c>
-      <c r="B11" s="35">
+      <c r="B11" s="33">
         <v>46275</v>
       </c>
-      <c r="C11" s="36">
+      <c r="C11" s="34">
         <v>46275</v>
       </c>
-      <c r="D11" s="34" t="s">
-        <v>35</v>
-      </c>
-      <c r="E11" s="34"/>
-      <c r="F11" s="38" t="s">
+      <c r="D11" s="32" t="s">
+        <v>34</v>
+      </c>
+      <c r="E11" s="32"/>
+      <c r="F11" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="34"/>
-    </row>
-    <row r="12" spans="1:7" s="32" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="29">
+      <c r="G11" s="32"/>
+    </row>
+    <row r="12" spans="1:7" s="30" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="27">
         <v>4</v>
       </c>
-      <c r="B12" s="30">
+      <c r="B12" s="28">
         <v>46279</v>
       </c>
-      <c r="C12" s="31">
+      <c r="C12" s="29">
         <v>46279</v>
       </c>
-      <c r="D12" s="29" t="s">
+      <c r="D12" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="E12" s="31"/>
-      <c r="F12" s="31"/>
-      <c r="G12" s="31"/>
-    </row>
-    <row r="13" spans="1:7" s="32" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="29">
+      <c r="E12" s="29"/>
+      <c r="F12" s="29"/>
+      <c r="G12" s="29"/>
+    </row>
+    <row r="13" spans="1:7" s="30" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="27">
         <v>4</v>
       </c>
-      <c r="B13" s="30">
+      <c r="B13" s="28">
         <v>46281</v>
       </c>
-      <c r="C13" s="31">
+      <c r="C13" s="29">
         <v>46281</v>
       </c>
-      <c r="D13" s="29" t="s">
+      <c r="D13" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="E13" s="31"/>
-      <c r="F13" s="31"/>
-      <c r="G13" s="31"/>
-    </row>
-    <row r="14" spans="1:7" s="32" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="29">
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
+      <c r="G13" s="29"/>
+    </row>
+    <row r="14" spans="1:7" s="30" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="27">
         <v>4</v>
       </c>
-      <c r="B14" s="30">
+      <c r="B14" s="28">
         <v>46282</v>
       </c>
-      <c r="C14" s="31">
+      <c r="C14" s="29">
         <v>46282</v>
       </c>
-      <c r="D14" s="29" t="s">
+      <c r="D14" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="E14" s="33"/>
-      <c r="F14" s="29"/>
-      <c r="G14" s="29"/>
+      <c r="E14" s="31"/>
+      <c r="F14" s="27"/>
+      <c r="G14" s="27"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="8">
@@ -878,22 +878,22 @@
       <c r="F16" s="10"/>
       <c r="G16" s="25"/>
     </row>
-    <row r="17" spans="1:7" s="37" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="34">
+    <row r="17" spans="1:7" s="35" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="32">
         <v>5</v>
       </c>
-      <c r="B17" s="35">
+      <c r="B17" s="33">
         <v>46289</v>
       </c>
-      <c r="C17" s="36">
+      <c r="C17" s="34">
         <v>46289</v>
       </c>
-      <c r="D17" s="34" t="s">
-        <v>37</v>
-      </c>
-      <c r="E17" s="34"/>
-      <c r="F17" s="38"/>
-      <c r="G17" s="34"/>
+      <c r="D17" s="32" t="s">
+        <v>36</v>
+      </c>
+      <c r="E17" s="32"/>
+      <c r="F17" s="36"/>
+      <c r="G17" s="32"/>
     </row>
     <row r="18" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
@@ -926,9 +926,6 @@
         <v>17</v>
       </c>
       <c r="E19" s="3"/>
-      <c r="F19" s="39" t="s">
-        <v>47</v>
-      </c>
       <c r="G19" s="5"/>
     </row>
     <row r="20" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -941,11 +938,11 @@
       <c r="C20" s="14">
         <v>46296</v>
       </c>
-      <c r="D20" s="34" t="s">
-        <v>38</v>
-      </c>
-      <c r="E20" s="34"/>
-      <c r="F20" s="38" t="s">
+      <c r="D20" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="E20" s="32"/>
+      <c r="F20" s="36" t="s">
         <v>18</v>
       </c>
       <c r="G20" s="12"/>
@@ -995,7 +992,7 @@
         <v>46303</v>
       </c>
       <c r="D23" s="12" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E23" s="15"/>
       <c r="F23" s="12"/>
@@ -1034,7 +1031,9 @@
       <c r="E25" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="F25" s="3"/>
+      <c r="F25" s="37" t="s">
+        <v>46</v>
+      </c>
       <c r="G25" s="5"/>
     </row>
     <row r="26" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1099,7 +1098,7 @@
         <v>46317</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E29" s="15"/>
       <c r="F29" s="26" t="s">
@@ -1154,7 +1153,7 @@
         <v>46324</v>
       </c>
       <c r="D32" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E32" s="15"/>
       <c r="F32" s="12"/>
@@ -1204,7 +1203,7 @@
         <v>46331</v>
       </c>
       <c r="D35" s="12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E35" s="15"/>
       <c r="F35" s="26" t="s">
@@ -1279,7 +1278,7 @@
       <c r="E39" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="F39" s="39" t="s">
+      <c r="F39" s="37" t="s">
         <v>27</v>
       </c>
       <c r="G39" s="5"/>
@@ -1312,7 +1311,7 @@
         <v>46345</v>
       </c>
       <c r="D41" s="12" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E41" s="15"/>
       <c r="F41" s="12"/>
@@ -1363,11 +1362,11 @@
         <v>46352</v>
       </c>
       <c r="D44" s="12" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E44" s="15"/>
       <c r="F44" s="26" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G44" s="12"/>
     </row>
@@ -1402,8 +1401,8 @@
         <v>33</v>
       </c>
       <c r="E46" s="23"/>
-      <c r="F46" s="40" t="s">
-        <v>34</v>
+      <c r="F46" s="38" t="s">
+        <v>48</v>
       </c>
       <c r="G46" s="23"/>
     </row>
@@ -1418,7 +1417,7 @@
         <v>46359</v>
       </c>
       <c r="D47" s="12" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E47" s="15"/>
       <c r="F47" s="12"/>

</xml_diff>

<commit_message>
Actualizar cronograma: clase del 14-oct suspendida y recuperación en semana 10
- 14-oct sin clase; se agrega clase de recuperación de Inferencia MCO en semana 10 (fecha por confirmar)
- 19-oct cierra Estimación MCO; Inferencia MCO parte el 21-oct
- Propuesta trabajo grupal pasa al 21-oct

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Cronograma_Analisis_Econometrico_2026.xlsx
+++ b/Cronograma_Analisis_Econometrico_2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ramirodeelejalde/Dropbox/Teaching/Econometria I_MAE/econometria_mae/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{999CF562-A876-1F40-AE4D-DDED07E37B6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF9493DA-685F-7749-8C97-4B01B7C83D22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7740" yWindow="1680" windowWidth="24860" windowHeight="15680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1140" yWindow="2080" windowWidth="24860" windowHeight="15680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cronograma" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="53">
   <si>
     <t>Semana</t>
   </si>
@@ -55,13 +55,25 @@
     <t>No hay ayudantía</t>
   </si>
   <si>
+    <t xml:space="preserve">Ayudante 2026: Alexis Silva. Horario por confirmar. </t>
+  </si>
+  <si>
     <t>Proyector lineal</t>
   </si>
   <si>
     <t>Tarea 1</t>
   </si>
   <si>
+    <t>Ayudantía 1: Repaso estadística, esperanza condicional, proyector lineal</t>
+  </si>
+  <si>
     <t>Teoría asintótica</t>
+  </si>
+  <si>
+    <t>Ayudantía 2: Control 1/ Solución tarea 1</t>
+  </si>
+  <si>
+    <t>Tarea 1 / Control 1</t>
   </si>
   <si>
     <t>Receso Académico</t>
@@ -70,22 +82,34 @@
     <t>Tarea 2</t>
   </si>
   <si>
-    <t>Tarea 1 / Control 1</t>
+    <t>Ayudantía 3: Teoría asintótica</t>
   </si>
   <si>
     <t>Estimación MCO</t>
   </si>
   <si>
+    <t>Ayudantía 4: Control 2/ Solución tarea 2</t>
+  </si>
+  <si>
     <t>Tarea 2 / Control 2</t>
+  </si>
+  <si>
+    <t>Prueba 1</t>
+  </si>
+  <si>
+    <t>Ayudantía 5: Estimación MCO</t>
   </si>
   <si>
     <t>FERIADO – Encuentro de Dos Mundos (sin clases)</t>
   </si>
   <si>
+    <t>Sin clase (se recupera)</t>
+  </si>
+  <si>
     <t>Tarea 3</t>
   </si>
   <si>
-    <t>Prueba 1</t>
+    <t>Clase suspendida; se recupera con clase adicional en semana 10. Propuesta trabajo grupal pasa al 21-oct.</t>
   </si>
   <si>
     <t>Ayudantía 6: Estimación MCO</t>
@@ -94,79 +118,67 @@
     <t>Inferencia MCO</t>
   </si>
   <si>
+    <t>Propuesta trabajo grupal</t>
+  </si>
+  <si>
+    <t>Ayudantía 7: Control 3/ Solución tarea 3</t>
+  </si>
+  <si>
     <t>Tarea 3 / Control 3</t>
+  </si>
+  <si>
+    <t>Tarea 4</t>
+  </si>
+  <si>
+    <t>Ayudantía 8: Inferencia MCO</t>
+  </si>
+  <si>
+    <t>Clase de recuperación: Inferencia MCO</t>
+  </si>
+  <si>
+    <t>Fecha y horario por confirmar</t>
   </si>
   <si>
     <t>Variables instrumentales (VI)</t>
   </si>
   <si>
-    <t>Tarea 4</t>
+    <t>Ayudantía 9: Control 4/ Solución tarea 4</t>
+  </si>
+  <si>
+    <t>Tarea 4 / Control 4</t>
+  </si>
+  <si>
+    <t>Prueba 2</t>
+  </si>
+  <si>
+    <t>Ayudantía 10: Variables instrumentales</t>
+  </si>
+  <si>
+    <t>Tarea 5</t>
   </si>
   <si>
     <t>Avance de Trabajo Grupal</t>
   </si>
   <si>
-    <t>Ayudantía 10: Variables instrumentales</t>
+    <t>Temas adicionales MCO</t>
   </si>
   <si>
-    <t>Prueba 2</t>
+    <t>Ayudantía 11: Variables instrumentales</t>
   </si>
   <si>
-    <t>Tarea 5</t>
+    <t>Ayudantía 12: Control 5/ Solución tarea 5</t>
   </si>
   <si>
-    <t>Tarea 4 / Control 4</t>
-  </si>
-  <si>
-    <t>Temas adicionales MCO</t>
+    <t>Tarea 5/ Control 5</t>
   </si>
   <si>
     <t xml:space="preserve">Presentación Trabajo Grupal </t>
   </si>
   <si>
-    <t>Ayudantía 2: Control 1/ Solución tarea 1</t>
-  </si>
-  <si>
-    <t>Ayudantía 1: Repaso estadística, esperanza condicional, proyector lineal</t>
-  </si>
-  <si>
-    <t>Ayudantía 3: Teoría asintótica</t>
-  </si>
-  <si>
-    <t>Ayudantía 4: Control 2/ Solución tarea 2</t>
-  </si>
-  <si>
-    <t>Ayudantía 5: Estimación MCO</t>
-  </si>
-  <si>
-    <t>Ayudantía 8: Inferencia MCO</t>
-  </si>
-  <si>
-    <t>Ayudantía 7: Control 3/ Solución tarea 3</t>
-  </si>
-  <si>
-    <t>Ayudantía 9: Control 4/ Solución tarea 4</t>
-  </si>
-  <si>
-    <t>Ayudantía 11: Variables instrumentales</t>
-  </si>
-  <si>
-    <t>Tarea 5/ Control 5</t>
-  </si>
-  <si>
-    <t>Ayudantía 12: Control 5/ Solución tarea 5</t>
+    <t>Trabajo Grupal/Presentación</t>
   </si>
   <si>
     <t>Ayudantía 13: Repaso</t>
-  </si>
-  <si>
-    <t>Propuesta trabajo grupal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ayudante 2026: Alexis Silva. Horario por confirmar. </t>
-  </si>
-  <si>
-    <t>Trabajo Grupal/Presentación</t>
   </si>
 </sst>
 </file>
@@ -324,7 +336,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -368,10 +380,12 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="3" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -599,38 +613,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="39" t="s">
+      <c r="B1" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="39" t="s">
+      <c r="C1" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="39" t="s">
+      <c r="D1" s="40" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1"/>
-      <c r="G1" s="39" t="s">
+      <c r="G1" s="40" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="40"/>
-      <c r="B2" s="40"/>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
+      <c r="A2" s="41"/>
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
       <c r="E2" s="2" t="s">
         <v>6</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="40"/>
+      <c r="G2" s="41"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="8">
@@ -682,7 +696,7 @@
       <c r="E5" s="6"/>
       <c r="F5" s="6"/>
       <c r="G5" s="7" t="s">
-        <v>47</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -696,7 +710,7 @@
         <v>46265</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
@@ -713,10 +727,10 @@
         <v>46267</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F7" s="5"/>
       <c r="G7" s="5"/>
@@ -732,7 +746,7 @@
         <v>46268</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="E8" s="15"/>
       <c r="F8" s="12"/>
@@ -749,7 +763,7 @@
         <v>46272</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E9" s="10"/>
       <c r="F9" s="10"/>
@@ -766,7 +780,7 @@
         <v>46274</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E10" s="10"/>
       <c r="F10" s="10"/>
@@ -783,11 +797,11 @@
         <v>46275</v>
       </c>
       <c r="D11" s="32" t="s">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="E11" s="32"/>
       <c r="F11" s="36" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G11" s="32"/>
     </row>
@@ -802,7 +816,7 @@
         <v>46279</v>
       </c>
       <c r="D12" s="27" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="E12" s="29"/>
       <c r="F12" s="29"/>
@@ -819,7 +833,7 @@
         <v>46281</v>
       </c>
       <c r="D13" s="27" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="E13" s="29"/>
       <c r="F13" s="29"/>
@@ -836,7 +850,7 @@
         <v>46282</v>
       </c>
       <c r="D14" s="27" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="E14" s="31"/>
       <c r="F14" s="27"/>
@@ -853,7 +867,7 @@
         <v>46286</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E15" s="10"/>
       <c r="F15" s="10"/>
@@ -870,10 +884,10 @@
         <v>46288</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F16" s="10"/>
       <c r="G16" s="25"/>
@@ -889,7 +903,7 @@
         <v>46289</v>
       </c>
       <c r="D17" s="32" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E17" s="32"/>
       <c r="F17" s="36"/>
@@ -906,7 +920,7 @@
         <v>46293</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
@@ -923,7 +937,7 @@
         <v>46295</v>
       </c>
       <c r="D19" s="19" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E19" s="3"/>
       <c r="G19" s="5"/>
@@ -939,11 +953,11 @@
         <v>46296</v>
       </c>
       <c r="D20" s="32" t="s">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="E20" s="32"/>
       <c r="F20" s="36" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="G20" s="12"/>
     </row>
@@ -958,7 +972,7 @@
         <v>46300</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
@@ -975,7 +989,7 @@
         <v>46302</v>
       </c>
       <c r="D22" s="24" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E22" s="21"/>
       <c r="F22" s="21"/>
@@ -992,7 +1006,7 @@
         <v>46303</v>
       </c>
       <c r="D23" s="12" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="E23" s="15"/>
       <c r="F23" s="12"/>
@@ -1009,7 +1023,7 @@
         <v>46307</v>
       </c>
       <c r="D24" s="19" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
@@ -1026,15 +1040,15 @@
         <v>46309</v>
       </c>
       <c r="D25" s="19" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F25" s="37" t="s">
-        <v>46</v>
-      </c>
-      <c r="G25" s="5"/>
+        <v>28</v>
+      </c>
+      <c r="F25" s="37"/>
+      <c r="G25" s="42" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="26" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="12">
@@ -1047,7 +1061,7 @@
         <v>46310</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="E26" s="15"/>
       <c r="F26" s="12"/>
@@ -1063,8 +1077,8 @@
       <c r="C27" s="10">
         <v>46314</v>
       </c>
-      <c r="D27" s="17" t="s">
-        <v>23</v>
+      <c r="D27" s="8" t="s">
+        <v>21</v>
       </c>
       <c r="E27" s="8"/>
       <c r="F27" s="8"/>
@@ -1080,11 +1094,13 @@
       <c r="C28" s="10">
         <v>46316</v>
       </c>
-      <c r="D28" s="8" t="s">
-        <v>23</v>
+      <c r="D28" s="17" t="s">
+        <v>31</v>
       </c>
       <c r="E28" s="8"/>
-      <c r="F28" s="8"/>
+      <c r="F28" s="39" t="s">
+        <v>32</v>
+      </c>
       <c r="G28" s="10"/>
     </row>
     <row r="29" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1098,11 +1114,11 @@
         <v>46317</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="E29" s="15"/>
       <c r="F29" s="26" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="G29" s="12"/>
     </row>
@@ -1117,7 +1133,7 @@
         <v>46321</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="E30" s="8"/>
       <c r="F30" s="8"/>
@@ -1134,10 +1150,10 @@
         <v>46323</v>
       </c>
       <c r="D31" s="8" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="F31" s="8"/>
       <c r="G31" s="10"/>
@@ -1153,284 +1169,290 @@
         <v>46324</v>
       </c>
       <c r="D32" s="12" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E32" s="15"/>
       <c r="F32" s="12"/>
       <c r="G32" s="12"/>
     </row>
     <row r="33" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="3">
-        <v>11</v>
-      </c>
-      <c r="B33" s="4">
-        <v>46328</v>
-      </c>
-      <c r="C33" s="5">
-        <v>46328</v>
-      </c>
-      <c r="D33" s="18" t="s">
-        <v>25</v>
-      </c>
-      <c r="E33" s="3"/>
-      <c r="G33" s="5"/>
+      <c r="A33" s="8">
+        <v>10</v>
+      </c>
+      <c r="B33" s="9"/>
+      <c r="C33" s="10"/>
+      <c r="D33" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="E33" s="8"/>
+      <c r="F33" s="8"/>
+      <c r="G33" s="25" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="34" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="3">
         <v>11</v>
       </c>
       <c r="B34" s="4">
+        <v>46328</v>
+      </c>
+      <c r="C34" s="5">
+        <v>46328</v>
+      </c>
+      <c r="D34" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="E34" s="3"/>
+      <c r="G34" s="5"/>
+    </row>
+    <row r="35" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="3">
+        <v>11</v>
+      </c>
+      <c r="B35" s="4">
         <v>46330</v>
       </c>
-      <c r="C34" s="5">
+      <c r="C35" s="5">
         <v>46330</v>
       </c>
-      <c r="D34" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="E34" s="3"/>
-      <c r="F34" s="3"/>
-      <c r="G34" s="5"/>
-    </row>
-    <row r="35" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="12">
+      <c r="D35" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="E35" s="3"/>
+      <c r="F35" s="3"/>
+      <c r="G35" s="5"/>
+    </row>
+    <row r="36" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="12">
         <v>11</v>
       </c>
-      <c r="B35" s="13">
+      <c r="B36" s="13">
         <v>46331</v>
       </c>
-      <c r="C35" s="14">
+      <c r="C36" s="14">
         <v>46331</v>
       </c>
-      <c r="D35" s="12" t="s">
+      <c r="D36" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E36" s="15"/>
+      <c r="F36" s="26" t="s">
         <v>41</v>
       </c>
-      <c r="E35" s="15"/>
-      <c r="F35" s="26" t="s">
-        <v>31</v>
-      </c>
-      <c r="G35" s="12"/>
-    </row>
-    <row r="36" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="3">
+      <c r="G36" s="12"/>
+    </row>
+    <row r="37" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="3">
         <v>12</v>
       </c>
-      <c r="B36" s="4">
+      <c r="B37" s="4">
         <v>46335</v>
       </c>
-      <c r="C36" s="5">
+      <c r="C37" s="5">
         <v>46335</v>
       </c>
-      <c r="D36" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="E36" s="3"/>
-      <c r="F36" s="3"/>
-      <c r="G36" s="5"/>
-    </row>
-    <row r="37" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="21">
+      <c r="D37" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="E37" s="3"/>
+      <c r="F37" s="3"/>
+      <c r="G37" s="5"/>
+    </row>
+    <row r="38" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="21">
         <v>12</v>
       </c>
-      <c r="B37" s="22">
+      <c r="B38" s="22">
         <v>46337</v>
       </c>
-      <c r="C37" s="23">
+      <c r="C38" s="23">
         <v>46337</v>
       </c>
-      <c r="D37" s="24" t="s">
-        <v>29</v>
-      </c>
-      <c r="E37" s="23"/>
-      <c r="F37" s="23"/>
-      <c r="G37" s="23"/>
-    </row>
-    <row r="38" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="12">
+      <c r="D38" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="E38" s="23"/>
+      <c r="F38" s="23"/>
+      <c r="G38" s="23"/>
+    </row>
+    <row r="39" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="12">
         <v>12</v>
       </c>
-      <c r="B38" s="13">
+      <c r="B39" s="13">
         <v>46338</v>
       </c>
-      <c r="C38" s="14">
+      <c r="C39" s="14">
         <v>46338</v>
       </c>
-      <c r="D38" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="E38" s="15"/>
-      <c r="F38" s="12"/>
-      <c r="G38" s="12"/>
-    </row>
-    <row r="39" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="3">
+      <c r="D39" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="E39" s="15"/>
+      <c r="F39" s="12"/>
+      <c r="G39" s="12"/>
+    </row>
+    <row r="40" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="3">
         <v>13</v>
       </c>
-      <c r="B39" s="4">
+      <c r="B40" s="4">
         <v>46342</v>
       </c>
-      <c r="C39" s="5">
+      <c r="C40" s="5">
         <v>46342</v>
       </c>
-      <c r="D39" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="E39" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="F39" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="G39" s="5"/>
-    </row>
-    <row r="40" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="8">
+      <c r="D40" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="F40" s="37" t="s">
+        <v>45</v>
+      </c>
+      <c r="G40" s="5"/>
+    </row>
+    <row r="41" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="8">
         <v>13</v>
       </c>
-      <c r="B40" s="9">
+      <c r="B41" s="9">
         <v>46344</v>
       </c>
-      <c r="C40" s="10">
+      <c r="C41" s="10">
         <v>46344</v>
       </c>
-      <c r="D40" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="E40" s="8"/>
-      <c r="F40" s="8"/>
-      <c r="G40" s="10"/>
-    </row>
-    <row r="41" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="12">
+      <c r="D41" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="E41" s="8"/>
+      <c r="F41" s="8"/>
+      <c r="G41" s="10"/>
+    </row>
+    <row r="42" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="12">
         <v>13</v>
       </c>
-      <c r="B41" s="13">
+      <c r="B42" s="13">
         <v>46345</v>
       </c>
-      <c r="C41" s="14">
+      <c r="C42" s="14">
         <v>46345</v>
       </c>
-      <c r="D41" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="E41" s="15"/>
-      <c r="F41" s="12"/>
-      <c r="G41" s="12"/>
-    </row>
-    <row r="42" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="8">
-        <v>14</v>
-      </c>
-      <c r="B42" s="9">
-        <v>46349</v>
-      </c>
-      <c r="C42" s="10">
-        <v>46349</v>
-      </c>
-      <c r="D42" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="E42" s="8"/>
-      <c r="F42" s="8"/>
-      <c r="G42" s="10"/>
+      <c r="D42" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="E42" s="15"/>
+      <c r="F42" s="12"/>
+      <c r="G42" s="12"/>
     </row>
     <row r="43" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="8">
         <v>14</v>
       </c>
       <c r="B43" s="9">
-        <v>46351</v>
+        <v>46349</v>
       </c>
       <c r="C43" s="10">
-        <v>46351</v>
+        <v>46349</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="E43" s="8"/>
       <c r="F43" s="8"/>
       <c r="G43" s="10"/>
     </row>
     <row r="44" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="12">
+      <c r="A44" s="8">
         <v>14</v>
       </c>
-      <c r="B44" s="13">
+      <c r="B44" s="9">
+        <v>46351</v>
+      </c>
+      <c r="C44" s="10">
+        <v>46351</v>
+      </c>
+      <c r="D44" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="E44" s="8"/>
+      <c r="F44" s="8"/>
+      <c r="G44" s="10"/>
+    </row>
+    <row r="45" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="12">
+        <v>14</v>
+      </c>
+      <c r="B45" s="13">
         <v>46352</v>
       </c>
-      <c r="C44" s="14">
+      <c r="C45" s="14">
         <v>46352</v>
       </c>
-      <c r="D44" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="E44" s="15"/>
-      <c r="F44" s="26" t="s">
-        <v>43</v>
-      </c>
-      <c r="G44" s="12"/>
-    </row>
-    <row r="45" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="8">
+      <c r="D45" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="E45" s="15"/>
+      <c r="F45" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="G45" s="12"/>
+    </row>
+    <row r="46" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="8">
         <v>15</v>
       </c>
-      <c r="B45" s="9">
+      <c r="B46" s="9">
         <v>46356</v>
       </c>
-      <c r="C45" s="10">
+      <c r="C46" s="10">
         <v>46356</v>
       </c>
-      <c r="D45" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="E45" s="8"/>
-      <c r="F45" s="8"/>
-      <c r="G45" s="10"/>
-    </row>
-    <row r="46" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="21">
+      <c r="D46" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="E46" s="8"/>
+      <c r="F46" s="8"/>
+      <c r="G46" s="10"/>
+    </row>
+    <row r="47" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="21">
         <v>15</v>
       </c>
-      <c r="B46" s="22">
+      <c r="B47" s="22">
         <v>46358</v>
       </c>
-      <c r="C46" s="23">
+      <c r="C47" s="23">
         <v>46358</v>
       </c>
-      <c r="D46" s="24" t="s">
-        <v>33</v>
-      </c>
-      <c r="E46" s="23"/>
-      <c r="F46" s="38" t="s">
-        <v>48</v>
-      </c>
-      <c r="G46" s="23"/>
-    </row>
-    <row r="47" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="12">
+      <c r="D47" s="24" t="s">
+        <v>50</v>
+      </c>
+      <c r="E47" s="23"/>
+      <c r="F47" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="G47" s="23"/>
+    </row>
+    <row r="48" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="12">
         <v>15</v>
       </c>
-      <c r="B47" s="13">
+      <c r="B48" s="13">
         <v>46359</v>
       </c>
-      <c r="C47" s="14">
+      <c r="C48" s="14">
         <v>46359</v>
       </c>
-      <c r="D47" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="E47" s="15"/>
-      <c r="F47" s="12"/>
-      <c r="G47" s="12"/>
-    </row>
-    <row r="48" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="20"/>
-      <c r="B48" s="20"/>
-      <c r="C48" s="20"/>
-      <c r="D48" s="20"/>
-      <c r="E48" s="20"/>
-      <c r="F48" s="20"/>
-      <c r="G48" s="20"/>
+      <c r="D48" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="E48" s="15"/>
+      <c r="F48" s="12"/>
+      <c r="G48" s="12"/>
     </row>
     <row r="49" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="20"/>
@@ -9856,7 +9878,15 @@
       <c r="F984" s="20"/>
       <c r="G984" s="20"/>
     </row>
-    <row r="985" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="985" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A985" s="20"/>
+      <c r="B985" s="20"/>
+      <c r="C985" s="20"/>
+      <c r="D985" s="20"/>
+      <c r="E985" s="20"/>
+      <c r="F985" s="20"/>
+      <c r="G985" s="20"/>
+    </row>
     <row r="986" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="987" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="988" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>

</xml_diff>